<commit_message>
@ chore(sync): working tree 전체 git 동기화 (미커밋 0)
prod = working tree 기준으로 git 일괄 반영. 개별 기능 설명은 직전 커밋들에 있음.
포함: 누적 소스/문서/e2e 스펙 + 빌드 산출물(dist2/dist3) + 이미지 에셋 + 옛 파일 정리(삭제).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/web/user/dist2/template_list (5).xlsx
+++ b/web/user/dist2/template_list (5).xlsx
@@ -125,22 +125,25 @@
     <t>앱링크</t>
   </si>
   <si>
-    <t>채팅상담요청알림</t>
+    <t>채팅응답하기</t>
   </si>
   <si>
     <t>sajuplan://#{url}</t>
   </si>
   <si>
-    <t>등록</t>
+    <t>승인</t>
   </si>
   <si>
     <t>발송전</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>2026-05-30 19:46:04</t>
+  </si>
+  <si>
+    <t>2026-05-30 20:03:42</t>
+  </si>
+  <si>
+    <t>2026-06-01 10:47:11</t>
   </si>
   <si>
     <t>settlement_complete</t>
@@ -160,6 +163,12 @@
     <t>2026-05-29 13:05:28</t>
   </si>
   <si>
+    <t>2026-05-30 20:03:43</t>
+  </si>
+  <si>
+    <t>2026-06-01 10:47:19</t>
+  </si>
+  <si>
     <t>chat_auto_cancelled_to_member</t>
   </si>
   <si>
@@ -173,9 +182,6 @@
 - 사주플랜</t>
   </si>
   <si>
-    <t>승인</t>
-  </si>
-  <si>
     <t>2026-05-23 18:26:56</t>
   </si>
   <si>
@@ -222,10 +228,7 @@
     <t>2026-05-23 13:32:54</t>
   </si>
   <si>
-    <t>2026-05-30 19:20:29</t>
-  </si>
-  <si>
-    <t>2026-05-29 11:42:16</t>
+    <t>2026-06-01 10:47:31</t>
   </si>
   <si>
     <t>payout_request_rejected</t>
@@ -310,13 +313,13 @@
     <t>후기 확인하기</t>
   </si>
   <si>
+    <t>정상</t>
+  </si>
+  <si>
     <t>2026-05-21 15:00:26</t>
   </si>
   <si>
-    <t>2026-05-30 19:20:30</t>
-  </si>
-  <si>
-    <t>2026-05-21 17:17:29</t>
+    <t>2026-06-01 10:47:50</t>
   </si>
   <si>
     <t>ops_admin_alert_v2</t>
@@ -329,9 +332,6 @@
 유형: #{category}
 시각: #{at}
 #{detail}</t>
-  </si>
-  <si>
-    <t>정상</t>
   </si>
   <si>
     <t>2026-05-21 14:59:15</t>
@@ -398,10 +398,10 @@
     <t>2026-05-21 14:55:26</t>
   </si>
   <si>
-    <t>2026-05-30 19:21:58</t>
-  </si>
-  <si>
-    <t>2026-05-21 17:20:25</t>
+    <t>2026-05-30 20:03:44</t>
+  </si>
+  <si>
+    <t>2026-06-01 10:48:13</t>
   </si>
   <si>
     <t>qa_ask_v2</t>
@@ -423,7 +423,7 @@
     <t>2026-05-21 14:54:14</t>
   </si>
   <si>
-    <t>2026-05-21 17:21:11</t>
+    <t>2026-06-01 10:48:32</t>
   </si>
   <si>
     <t>qa_answer_v2</t>
@@ -444,7 +444,7 @@
     <t>2026-05-21 14:52:48</t>
   </si>
   <si>
-    <t>2026-05-21 17:21:33</t>
+    <t>2026-06-01 10:48:42</t>
   </si>
   <si>
     <t>chat_counseling_v2</t>
@@ -465,10 +465,10 @@
     <t>2026-05-21 14:49:11</t>
   </si>
   <si>
-    <t>2026-05-30 19:20:32</t>
-  </si>
-  <si>
-    <t>2026-05-21 16:55:31</t>
+    <t>2026-05-30 20:03:45</t>
+  </si>
+  <si>
+    <t>2026-06-01 10:48:54</t>
   </si>
 </sst>
 </file>
@@ -1067,16 +1067,16 @@
         <v>38</v>
       </c>
       <c r="AR3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AS3" s="1" t="s">
+      <c r="AT3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AT3" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="AU3" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:47">
@@ -1084,16 +1084,16 @@
         <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>33</v>
@@ -1105,16 +1105,16 @@
         <v>38</v>
       </c>
       <c r="AR4" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AS4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AT4" s="1" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="AU4" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:47">
@@ -1122,37 +1122,37 @@
         <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AQ5" s="1" t="s">
         <v>38</v>
       </c>
       <c r="AR5" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS5" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AT5" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AU5" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:47">
@@ -1175,34 +1175,34 @@
         <v>33</v>
       </c>
       <c r="L6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AP6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AQ6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AR6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AT6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AP6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AQ6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AR6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AS6" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT6" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="AU6" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:47">
@@ -1210,16 +1210,16 @@
         <v>28</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>33</v>
@@ -1228,7 +1228,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -1243,16 +1243,16 @@
         <v>38</v>
       </c>
       <c r="AR7" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS7" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AT7" s="1" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="AU7" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:47">
@@ -1260,37 +1260,37 @@
         <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AQ8" s="1" t="s">
         <v>38</v>
       </c>
       <c r="AR8" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS8" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AT8" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AU8" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:47">
@@ -1298,37 +1298,37 @@
         <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>33</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AQ9" s="1" t="s">
         <v>38</v>
       </c>
       <c r="AR9" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AT9" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AU9" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:47">
@@ -1336,37 +1336,37 @@
         <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>33</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AQ10" s="1" t="s">
         <v>38</v>
       </c>
       <c r="AR10" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS10" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AT10" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AU10" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:47">
@@ -1374,16 +1374,16 @@
         <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>33</v>
@@ -1392,7 +1392,7 @@
         <v>34</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>36</v>
@@ -1404,19 +1404,19 @@
         <v>37</v>
       </c>
       <c r="AQ11" s="1" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="AR11" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS11" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AT11" s="1" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="AU11" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:47">
@@ -1424,28 +1424,28 @@
         <v>28</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>33</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AQ12" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="AR12" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS12" s="1" t="s">
         <v>93</v>
@@ -1477,7 +1477,7 @@
         <v>33</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>99</v>
@@ -1545,7 +1545,7 @@
         <v>38</v>
       </c>
       <c r="AR14" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS14" s="1" t="s">
         <v>109</v>
@@ -1592,16 +1592,16 @@
         <v>37</v>
       </c>
       <c r="AQ15" s="1" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="AR15" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS15" s="1" t="s">
         <v>116</v>
       </c>
       <c r="AT15" s="1" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="AU15" s="1" t="s">
         <v>117</v>
@@ -1645,13 +1645,13 @@
         <v>38</v>
       </c>
       <c r="AR16" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS16" s="1" t="s">
         <v>122</v>
       </c>
       <c r="AT16" s="1" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="AU16" s="1" t="s">
         <v>123</v>
@@ -1695,7 +1695,7 @@
         <v>38</v>
       </c>
       <c r="AR17" s="1" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="AS17" s="1" t="s">
         <v>128</v>

</xml_diff>